<commit_message>
Instagram + Facebook: 2 Reels a day (one per live book); Benny Reel is now a must on Tuesday
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/campaigns/2026-10-06/POSTING-PLAN-Tue-Oct-6.xlsx
+++ b/campaigns/2026-10-06/POSTING-PLAN-Tue-Oct-6.xlsx
@@ -578,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -658,27 +658,27 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A6,$D$16:$D$26,"Video",$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A6,$D$16:$D$28,"Video",$I$16:$I$28,"Must")</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A6,$D$16:$D$26,"Video",$I$16:$I$26,"Optional")</f>
+        <f>COUNTIFS($C$16:$C$28,$A6,$D$16:$D$28,"Video",$I$16:$I$28,"Optional")</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A6,$D$16:$D$26,"Carousel")</f>
+        <f>COUNTIFS($C$16:$C$28,$A6,$D$16:$D$28,"Carousel")</f>
         <v/>
       </c>
       <c r="E6" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A6,$D$16:$D$26,"Pin")</f>
+        <f>COUNTIFS($C$16:$C$28,$A6,$D$16:$D$28,"Pin")</f>
         <v/>
       </c>
       <c r="F6" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A6,$D$16:$D$26,"Story")</f>
+        <f>COUNTIFS($C$16:$C$28,$A6,$D$16:$D$28,"Story")</f>
         <v/>
       </c>
       <c r="G6" s="7">
-        <f>COUNTIFS($C$16:$C$26,$A6,$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A6,$I$16:$I$28,"Must")</f>
         <v/>
       </c>
     </row>
@@ -689,27 +689,27 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A7,$D$16:$D$26,"Video",$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A7,$D$16:$D$28,"Video",$I$16:$I$28,"Must")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A7,$D$16:$D$26,"Video",$I$16:$I$26,"Optional")</f>
+        <f>COUNTIFS($C$16:$C$28,$A7,$D$16:$D$28,"Video",$I$16:$I$28,"Optional")</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A7,$D$16:$D$26,"Carousel")</f>
+        <f>COUNTIFS($C$16:$C$28,$A7,$D$16:$D$28,"Carousel")</f>
         <v/>
       </c>
       <c r="E7" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A7,$D$16:$D$26,"Pin")</f>
+        <f>COUNTIFS($C$16:$C$28,$A7,$D$16:$D$28,"Pin")</f>
         <v/>
       </c>
       <c r="F7" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A7,$D$16:$D$26,"Story")</f>
+        <f>COUNTIFS($C$16:$C$28,$A7,$D$16:$D$28,"Story")</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>COUNTIFS($C$16:$C$26,$A7,$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A7,$I$16:$I$28,"Must")</f>
         <v/>
       </c>
     </row>
@@ -720,27 +720,27 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A8,$D$16:$D$26,"Video",$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A8,$D$16:$D$28,"Video",$I$16:$I$28,"Must")</f>
         <v/>
       </c>
       <c r="C8" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A8,$D$16:$D$26,"Video",$I$16:$I$26,"Optional")</f>
+        <f>COUNTIFS($C$16:$C$28,$A8,$D$16:$D$28,"Video",$I$16:$I$28,"Optional")</f>
         <v/>
       </c>
       <c r="D8" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A8,$D$16:$D$26,"Carousel")</f>
+        <f>COUNTIFS($C$16:$C$28,$A8,$D$16:$D$28,"Carousel")</f>
         <v/>
       </c>
       <c r="E8" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A8,$D$16:$D$26,"Pin")</f>
+        <f>COUNTIFS($C$16:$C$28,$A8,$D$16:$D$28,"Pin")</f>
         <v/>
       </c>
       <c r="F8" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A8,$D$16:$D$26,"Story")</f>
+        <f>COUNTIFS($C$16:$C$28,$A8,$D$16:$D$28,"Story")</f>
         <v/>
       </c>
       <c r="G8" s="7">
-        <f>COUNTIFS($C$16:$C$26,$A8,$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A8,$I$16:$I$28,"Must")</f>
         <v/>
       </c>
     </row>
@@ -751,27 +751,27 @@
         </is>
       </c>
       <c r="B9" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A9,$D$16:$D$26,"Video",$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A9,$D$16:$D$28,"Video",$I$16:$I$28,"Must")</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A9,$D$16:$D$26,"Video",$I$16:$I$26,"Optional")</f>
+        <f>COUNTIFS($C$16:$C$28,$A9,$D$16:$D$28,"Video",$I$16:$I$28,"Optional")</f>
         <v/>
       </c>
       <c r="D9" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A9,$D$16:$D$26,"Carousel")</f>
+        <f>COUNTIFS($C$16:$C$28,$A9,$D$16:$D$28,"Carousel")</f>
         <v/>
       </c>
       <c r="E9" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A9,$D$16:$D$26,"Pin")</f>
+        <f>COUNTIFS($C$16:$C$28,$A9,$D$16:$D$28,"Pin")</f>
         <v/>
       </c>
       <c r="F9" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A9,$D$16:$D$26,"Story")</f>
+        <f>COUNTIFS($C$16:$C$28,$A9,$D$16:$D$28,"Story")</f>
         <v/>
       </c>
       <c r="G9" s="7">
-        <f>COUNTIFS($C$16:$C$26,$A9,$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A9,$I$16:$I$28,"Must")</f>
         <v/>
       </c>
     </row>
@@ -782,27 +782,27 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A10,$D$16:$D$26,"Video",$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A10,$D$16:$D$28,"Video",$I$16:$I$28,"Must")</f>
         <v/>
       </c>
       <c r="C10" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A10,$D$16:$D$26,"Video",$I$16:$I$26,"Optional")</f>
+        <f>COUNTIFS($C$16:$C$28,$A10,$D$16:$D$28,"Video",$I$16:$I$28,"Optional")</f>
         <v/>
       </c>
       <c r="D10" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A10,$D$16:$D$26,"Carousel")</f>
+        <f>COUNTIFS($C$16:$C$28,$A10,$D$16:$D$28,"Carousel")</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A10,$D$16:$D$26,"Pin")</f>
+        <f>COUNTIFS($C$16:$C$28,$A10,$D$16:$D$28,"Pin")</f>
         <v/>
       </c>
       <c r="F10" s="6">
-        <f>COUNTIFS($C$16:$C$26,$A10,$D$16:$D$26,"Story")</f>
+        <f>COUNTIFS($C$16:$C$28,$A10,$D$16:$D$28,"Story")</f>
         <v/>
       </c>
       <c r="G10" s="7">
-        <f>COUNTIFS($C$16:$C$26,$A10,$I$16:$I$26,"Must")</f>
+        <f>COUNTIFS($C$16:$C$28,$A10,$I$16:$I$28,"Must")</f>
         <v/>
       </c>
     </row>
@@ -847,7 +847,7 @@
     <row r="13">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>Instagram + Facebook: post once in Meta Business Suite with both accounts ticked (counts as 1 Reel on each). Posting times are Czech time (= US afternoon).</t>
+          <t>Instagram + Facebook: 2 Reels a day, one per live book. Post each once in Meta Business Suite with both accounts ticked. Times are Czech time (= US afternoon).</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>instagram-facebook/2-OPTIONAL-benny-find-bella.mp4</t>
+          <t>instagram-facebook/2-benny-find-bella.mp4</t>
         </is>
       </c>
       <c r="H25" s="15" t="inlineStr">
@@ -1363,9 +1363,9 @@
           <t>instagram-facebook/CAPTIONS.md</t>
         </is>
       </c>
-      <c r="I25" s="22" t="inlineStr">
-        <is>
-          <t>Optional</t>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="J25" s="15" t="inlineStr"/>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
-          <t>instagram-facebook/2-OPTIONAL-benny-find-bella.mp4</t>
+          <t>instagram-facebook/2-benny-find-bella.mp4</t>
         </is>
       </c>
       <c r="H26" s="15" t="inlineStr">
@@ -1409,12 +1409,104 @@
           <t>instagram-facebook/CAPTIONS.md</t>
         </is>
       </c>
-      <c r="I26" s="22" t="inlineStr">
-        <is>
-          <t>Optional</t>
+      <c r="I26" s="17" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="J26" s="15" t="inlineStr"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>Share the Benny Reel + Link sticker to Amazon</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>Benny</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>(share the Reel you just posted)</t>
+        </is>
+      </c>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>instagram-facebook/CAPTIONS.md (Story steps)</t>
+        </is>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="J27" s="15" t="inlineStr"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>Share the Benny Reel + link to Amazon</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>Benny</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="inlineStr">
+        <is>
+          <t>(share the Reel you just posted)</t>
+        </is>
+      </c>
+      <c r="H28" s="15" t="inlineStr">
+        <is>
+          <t>instagram-facebook/CAPTIONS.md (Story steps)</t>
+        </is>
+      </c>
+      <c r="I28" s="17" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="J28" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>